<commit_message>
Own series: blank starter files for E1/E2 (extract from the records first); draft README, guide and notes record the decision
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction draft - own series OWN (from manuscript, not chart-checked).xlsx
+++ b/Extraction draft - own series OWN (from manuscript, not chart-checked).xlsx
@@ -638,10 +638,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>• 如果两位提取员宁可从这份草稿出发，逐格核对病历：可以，但这 5 例就不再是独立双人提取（先看到草稿会影响自己的判断），要在 Methods 里说明。这一点请三位在开始前定下，不要事后再改。</t>
+          <t>• 2026 年 10 月 18 日作者决定：按上面的建议，两位提取员先从病历独立提取，空白起始文件在 `search/extraction/own_series/`（`extraction_E1_OWN_starter.xlsx`、`extraction_E2_OWN_starter.xlsx`）。卞红强是否已知道这一决定没有确认。若改为从草稿出发逐格核对，这 5 例就不再是独立双人提取，要在 Methods 里说明，且应事先由三位定下。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Delete the extraction time log (EX_time_log) from workbook, scripts and extraction guide
Facts only, no reason recorded; protocol unchanged (it never described this log).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction draft - own series OWN (from manuscript, not chart-checked).xlsx
+++ b/Extraction draft - own series OWN (from manuscript, not chart-checked).xlsx
@@ -11,10 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart_check" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX_time_log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duration_calc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -716,21 +715,19 @@
       </c>
     </row>
     <row r="17" ht="18" customHeight="1"/>
-    <row r="18" ht="18" customHeight="1"/>
-    <row r="19" ht="36" customHeight="1"/>
+    <row r="18" ht="54" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
     <row r="20" ht="18" customHeight="1"/>
     <row r="21" ht="18" customHeight="1"/>
-    <row r="22" ht="18" customHeight="1"/>
-    <row r="23" ht="18" customHeight="1"/>
-    <row r="24" ht="36" customHeight="1"/>
-    <row r="25" ht="36" customHeight="1"/>
-    <row r="26" ht="54" customHeight="1"/>
-    <row r="27" ht="54" customHeight="1"/>
+    <row r="22" ht="36" customHeight="1"/>
+    <row r="23" ht="36" customHeight="1"/>
+    <row r="24" ht="54" customHeight="1"/>
+    <row r="25" ht="54" customHeight="1"/>
+    <row r="26" ht="36" customHeight="1"/>
+    <row r="27" ht="36" customHeight="1"/>
     <row r="28" ht="36" customHeight="1"/>
-    <row r="29" ht="36" customHeight="1"/>
-    <row r="30" ht="36" customHeight="1"/>
-    <row r="31" ht="18" customHeight="1"/>
-    <row r="32" ht="54" customHeight="1"/>
+    <row r="29" ht="18" customHeight="1"/>
+    <row r="30" ht="54" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -37923,1052 +37920,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002F75B5"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G303"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>extractor</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>start</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>end</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>n_reports</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>n_patients</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="62" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Extractor</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Session start</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Session end</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Reports worked on</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Patients entered</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>yyyy-mm-dd</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>E1 = 舒俊，E2 = 卞红强</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>开始时间 hh:mm（本地时间）</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>结束时间 hh:mm</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>这一段时间处理了多少篇报告（整数）</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>这一段时间录入了多少名患者（整数）</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>例如中断原因、遇到的疑问</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="8" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="8" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="8" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="8" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="8" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="8" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="8" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="8" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="8" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="8" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="8" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="8" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="8" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="8" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="8" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="8" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="8" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="8" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="8" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="8" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="8" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="8" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="8" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="8" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="8" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="8" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="8" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="8" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="8" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="8" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="8" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="8" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="8" t="n"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="8" t="n"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="8" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="8" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="8" t="n"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="8" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="8" t="n"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="n"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="8" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="n"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="8" t="n"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="8" t="n"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="8" t="n"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="8" t="n"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="8" t="n"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="8" t="n"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="n"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="n"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="n"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="n"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="n"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="8" t="n"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="8" t="n"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="8" t="n"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="8" t="n"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="8" t="n"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="8" t="n"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="8" t="n"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="8" t="n"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="8" t="n"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="8" t="n"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="8" t="n"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="8" t="n"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="8" t="n"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="8" t="n"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="8" t="n"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="8" t="n"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="8" t="n"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="8" t="n"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="8" t="n"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="8" t="n"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="8" t="n"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="8" t="n"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="8" t="n"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="8" t="n"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="8" t="n"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="8" t="n"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="8" t="n"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="8" t="n"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="8" t="n"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="8" t="n"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="8" t="n"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="8" t="n"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="8" t="n"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="8" t="n"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="8" t="n"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="8" t="n"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="8" t="n"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="8" t="n"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="8" t="n"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="8" t="n"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="8" t="n"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="8" t="n"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="8" t="n"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="8" t="n"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="8" t="n"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="8" t="n"/>
-    </row>
-    <row r="178">
-      <c r="A178" s="8" t="n"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="8" t="n"/>
-    </row>
-    <row r="180">
-      <c r="A180" s="8" t="n"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="8" t="n"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="8" t="n"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="8" t="n"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="8" t="n"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="8" t="n"/>
-    </row>
-    <row r="186">
-      <c r="A186" s="8" t="n"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="8" t="n"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="8" t="n"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="8" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="8" t="n"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="8" t="n"/>
-    </row>
-    <row r="192">
-      <c r="A192" s="8" t="n"/>
-    </row>
-    <row r="193">
-      <c r="A193" s="8" t="n"/>
-    </row>
-    <row r="194">
-      <c r="A194" s="8" t="n"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="8" t="n"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="8" t="n"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="8" t="n"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="8" t="n"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="8" t="n"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="8" t="n"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="8" t="n"/>
-    </row>
-    <row r="202">
-      <c r="A202" s="8" t="n"/>
-    </row>
-    <row r="203">
-      <c r="A203" s="8" t="n"/>
-    </row>
-    <row r="204">
-      <c r="A204" s="8" t="n"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="8" t="n"/>
-    </row>
-    <row r="206">
-      <c r="A206" s="8" t="n"/>
-    </row>
-    <row r="207">
-      <c r="A207" s="8" t="n"/>
-    </row>
-    <row r="208">
-      <c r="A208" s="8" t="n"/>
-    </row>
-    <row r="209">
-      <c r="A209" s="8" t="n"/>
-    </row>
-    <row r="210">
-      <c r="A210" s="8" t="n"/>
-    </row>
-    <row r="211">
-      <c r="A211" s="8" t="n"/>
-    </row>
-    <row r="212">
-      <c r="A212" s="8" t="n"/>
-    </row>
-    <row r="213">
-      <c r="A213" s="8" t="n"/>
-    </row>
-    <row r="214">
-      <c r="A214" s="8" t="n"/>
-    </row>
-    <row r="215">
-      <c r="A215" s="8" t="n"/>
-    </row>
-    <row r="216">
-      <c r="A216" s="8" t="n"/>
-    </row>
-    <row r="217">
-      <c r="A217" s="8" t="n"/>
-    </row>
-    <row r="218">
-      <c r="A218" s="8" t="n"/>
-    </row>
-    <row r="219">
-      <c r="A219" s="8" t="n"/>
-    </row>
-    <row r="220">
-      <c r="A220" s="8" t="n"/>
-    </row>
-    <row r="221">
-      <c r="A221" s="8" t="n"/>
-    </row>
-    <row r="222">
-      <c r="A222" s="8" t="n"/>
-    </row>
-    <row r="223">
-      <c r="A223" s="8" t="n"/>
-    </row>
-    <row r="224">
-      <c r="A224" s="8" t="n"/>
-    </row>
-    <row r="225">
-      <c r="A225" s="8" t="n"/>
-    </row>
-    <row r="226">
-      <c r="A226" s="8" t="n"/>
-    </row>
-    <row r="227">
-      <c r="A227" s="8" t="n"/>
-    </row>
-    <row r="228">
-      <c r="A228" s="8" t="n"/>
-    </row>
-    <row r="229">
-      <c r="A229" s="8" t="n"/>
-    </row>
-    <row r="230">
-      <c r="A230" s="8" t="n"/>
-    </row>
-    <row r="231">
-      <c r="A231" s="8" t="n"/>
-    </row>
-    <row r="232">
-      <c r="A232" s="8" t="n"/>
-    </row>
-    <row r="233">
-      <c r="A233" s="8" t="n"/>
-    </row>
-    <row r="234">
-      <c r="A234" s="8" t="n"/>
-    </row>
-    <row r="235">
-      <c r="A235" s="8" t="n"/>
-    </row>
-    <row r="236">
-      <c r="A236" s="8" t="n"/>
-    </row>
-    <row r="237">
-      <c r="A237" s="8" t="n"/>
-    </row>
-    <row r="238">
-      <c r="A238" s="8" t="n"/>
-    </row>
-    <row r="239">
-      <c r="A239" s="8" t="n"/>
-    </row>
-    <row r="240">
-      <c r="A240" s="8" t="n"/>
-    </row>
-    <row r="241">
-      <c r="A241" s="8" t="n"/>
-    </row>
-    <row r="242">
-      <c r="A242" s="8" t="n"/>
-    </row>
-    <row r="243">
-      <c r="A243" s="8" t="n"/>
-    </row>
-    <row r="244">
-      <c r="A244" s="8" t="n"/>
-    </row>
-    <row r="245">
-      <c r="A245" s="8" t="n"/>
-    </row>
-    <row r="246">
-      <c r="A246" s="8" t="n"/>
-    </row>
-    <row r="247">
-      <c r="A247" s="8" t="n"/>
-    </row>
-    <row r="248">
-      <c r="A248" s="8" t="n"/>
-    </row>
-    <row r="249">
-      <c r="A249" s="8" t="n"/>
-    </row>
-    <row r="250">
-      <c r="A250" s="8" t="n"/>
-    </row>
-    <row r="251">
-      <c r="A251" s="8" t="n"/>
-    </row>
-    <row r="252">
-      <c r="A252" s="8" t="n"/>
-    </row>
-    <row r="253">
-      <c r="A253" s="8" t="n"/>
-    </row>
-    <row r="254">
-      <c r="A254" s="8" t="n"/>
-    </row>
-    <row r="255">
-      <c r="A255" s="8" t="n"/>
-    </row>
-    <row r="256">
-      <c r="A256" s="8" t="n"/>
-    </row>
-    <row r="257">
-      <c r="A257" s="8" t="n"/>
-    </row>
-    <row r="258">
-      <c r="A258" s="8" t="n"/>
-    </row>
-    <row r="259">
-      <c r="A259" s="8" t="n"/>
-    </row>
-    <row r="260">
-      <c r="A260" s="8" t="n"/>
-    </row>
-    <row r="261">
-      <c r="A261" s="8" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="8" t="n"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="8" t="n"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="8" t="n"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="8" t="n"/>
-    </row>
-    <row r="266">
-      <c r="A266" s="8" t="n"/>
-    </row>
-    <row r="267">
-      <c r="A267" s="8" t="n"/>
-    </row>
-    <row r="268">
-      <c r="A268" s="8" t="n"/>
-    </row>
-    <row r="269">
-      <c r="A269" s="8" t="n"/>
-    </row>
-    <row r="270">
-      <c r="A270" s="8" t="n"/>
-    </row>
-    <row r="271">
-      <c r="A271" s="8" t="n"/>
-    </row>
-    <row r="272">
-      <c r="A272" s="8" t="n"/>
-    </row>
-    <row r="273">
-      <c r="A273" s="8" t="n"/>
-    </row>
-    <row r="274">
-      <c r="A274" s="8" t="n"/>
-    </row>
-    <row r="275">
-      <c r="A275" s="8" t="n"/>
-    </row>
-    <row r="276">
-      <c r="A276" s="8" t="n"/>
-    </row>
-    <row r="277">
-      <c r="A277" s="8" t="n"/>
-    </row>
-    <row r="278">
-      <c r="A278" s="8" t="n"/>
-    </row>
-    <row r="279">
-      <c r="A279" s="8" t="n"/>
-    </row>
-    <row r="280">
-      <c r="A280" s="8" t="n"/>
-    </row>
-    <row r="281">
-      <c r="A281" s="8" t="n"/>
-    </row>
-    <row r="282">
-      <c r="A282" s="8" t="n"/>
-    </row>
-    <row r="283">
-      <c r="A283" s="8" t="n"/>
-    </row>
-    <row r="284">
-      <c r="A284" s="8" t="n"/>
-    </row>
-    <row r="285">
-      <c r="A285" s="8" t="n"/>
-    </row>
-    <row r="286">
-      <c r="A286" s="8" t="n"/>
-    </row>
-    <row r="287">
-      <c r="A287" s="8" t="n"/>
-    </row>
-    <row r="288">
-      <c r="A288" s="8" t="n"/>
-    </row>
-    <row r="289">
-      <c r="A289" s="8" t="n"/>
-    </row>
-    <row r="290">
-      <c r="A290" s="8" t="n"/>
-    </row>
-    <row r="291">
-      <c r="A291" s="8" t="n"/>
-    </row>
-    <row r="292">
-      <c r="A292" s="8" t="n"/>
-    </row>
-    <row r="293">
-      <c r="A293" s="8" t="n"/>
-    </row>
-    <row r="294">
-      <c r="A294" s="8" t="n"/>
-    </row>
-    <row r="295">
-      <c r="A295" s="8" t="n"/>
-    </row>
-    <row r="296">
-      <c r="A296" s="8" t="n"/>
-    </row>
-    <row r="297">
-      <c r="A297" s="8" t="n"/>
-    </row>
-    <row r="298">
-      <c r="A298" s="8" t="n"/>
-    </row>
-    <row r="299">
-      <c r="A299" s="8" t="n"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="8" t="n"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="8" t="n"/>
-    </row>
-    <row r="302">
-      <c r="A302" s="8" t="n"/>
-    </row>
-    <row r="303">
-      <c r="A303" s="8" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="B4:B303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
-      <formula1>Lists!$X$2:$X$4</formula1>
-    </dataValidation>
-    <dataValidation sqref="E4:E303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="F4:F303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Integer" error="请填非负整数。" type="whole" errorStyle="warning" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="007F7F7F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -39282,7 +38233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007F7F7F"/>
@@ -39958,14 +38909,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BBBBBB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AF11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39998,6 +38949,8 @@
     <col width="40" customWidth="1" min="28" max="28"/>
     <col width="37" customWidth="1" min="29" max="29"/>
     <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -40151,6 +39104,16 @@
           <t>ipd_received</t>
         </is>
       </c>
+      <c r="AE1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_delivery</t>
+        </is>
+      </c>
+      <c r="AF1" s="17" t="inlineStr">
+        <is>
+          <t>ipd_reached</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -40303,6 +39266,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Not yet sent</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -40455,6 +39428,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Sent, no bounce</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -40592,6 +39575,16 @@
           <t>Partial</t>
         </is>
       </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Bounced</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="F5" t="inlineStr">
@@ -40677,6 +39670,11 @@
       <c r="AC5" t="inlineStr">
         <is>
           <t>Not eligible after check</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>No address found</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Extraction workbook: add NR to presentation (template v2026-10-25a, guide v2026-10-25c); log author's answers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/Extraction draft - own series OWN (from manuscript, not chart-checked).xlsx
+++ b/Extraction draft - own series OWN (from manuscript, not chart-checked).xlsx
@@ -8158,7 +8158,7 @@
       </c>
       <c r="X3" s="7" t="inlineStr">
         <is>
-          <t>Acute / Chronic or intermittent / Acute on chronic / Asymptomatic / Mass only</t>
+          <t>Acute / Chronic or intermittent / Acute on chronic / Asymptomatic / Mass only；报告没写发作形式填 NR</t>
         </is>
       </c>
       <c r="Y3" s="7" t="inlineStr">
@@ -37811,7 +37811,7 @@
       <formula1>Lists!$I$2:$I$6</formula1>
     </dataValidation>
     <dataValidation sqref="X4:X1503" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in list" error="值不在列表里。请从下拉列表选择；确需例外请在 Notes 里说明。" type="list" errorStyle="warning">
-      <formula1>Lists!$J$2:$J$6</formula1>
+      <formula1>Lists!$J$2:$J$7</formula1>
     </dataValidation>
     <dataValidation sqref="Z4:Z1503" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Number or NR" error="请填数字；报告里没有请填 NR。" type="custom" errorStyle="warning">
       <formula1>OR(ISNUMBER(Z4),Z4="NR")</formula1>
@@ -39741,6 +39741,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>No operation</t>

</xml_diff>